<commit_message>
started medium array questions
</commit_message>
<xml_diff>
--- a/DSA for PLACEMENTS 1.xlsx
+++ b/DSA for PLACEMENTS 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9765abdd1e291f17/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_2E2C462B86E80A008A522AE716C952C441A6BCAD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B004C84D-FC14-48E7-A0E3-EFE78325CDA3}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_2E2C462B86E80A008A522AE716C952C441A6BCAD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C477E00-8E0D-439C-8DE7-BC490CEC3492}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="421">
   <si>
     <t>Do NOT send any edit request to this sheet. Instead, make a copy of your own.</t>
   </si>
@@ -1534,21 +1534,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1786,7 +1786,7 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="31" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="29"/>
@@ -1799,13 +1799,13 @@
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="32" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="29"/>
       <c r="F2" s="29"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="31" t="s">
+      <c r="H2" s="33" t="s">
         <v>2</v>
       </c>
       <c r="I2" s="29"/>
@@ -1861,7 +1861,7 @@
       <c r="I5" s="3"/>
     </row>
     <row r="6" spans="1:10" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="28" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="3" t="b">
@@ -2065,6 +2065,9 @@
       </c>
       <c r="H13" s="9"/>
       <c r="I13" s="3"/>
+      <c r="J13" s="1" t="s">
+        <v>419</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="14.5" x14ac:dyDescent="0.4">
       <c r="A14" s="29"/>
@@ -2090,6 +2093,9 @@
         <v>30</v>
       </c>
       <c r="I14" s="3"/>
+      <c r="J14" s="1" t="s">
+        <v>419</v>
+      </c>
     </row>
     <row r="15" spans="1:10" ht="14.5" x14ac:dyDescent="0.4">
       <c r="A15" s="29"/>
@@ -2554,7 +2560,7 @@
       <c r="I34" s="3"/>
     </row>
     <row r="35" spans="1:9" ht="15" x14ac:dyDescent="0.4">
-      <c r="A35" s="33" t="s">
+      <c r="A35" s="30" t="s">
         <v>68</v>
       </c>
       <c r="B35" s="3" t="b">
@@ -2745,7 +2751,7 @@
       <c r="I43" s="3"/>
     </row>
     <row r="44" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A44" s="32" t="s">
+      <c r="A44" s="28" t="s">
         <v>80</v>
       </c>
       <c r="B44" s="3" t="b">
@@ -3018,7 +3024,7 @@
       <c r="I56" s="3"/>
     </row>
     <row r="57" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A57" s="33" t="s">
+      <c r="A57" s="30" t="s">
         <v>98</v>
       </c>
       <c r="B57" s="3" t="b">
@@ -3307,7 +3313,7 @@
       <c r="I69" s="3"/>
     </row>
     <row r="70" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A70" s="33" t="s">
+      <c r="A70" s="30" t="s">
         <v>118</v>
       </c>
       <c r="B70" s="3" t="b">
@@ -3648,7 +3654,7 @@
       <c r="I84" s="3"/>
     </row>
     <row r="85" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A85" s="32" t="s">
+      <c r="A85" s="28" t="s">
         <v>145</v>
       </c>
       <c r="B85" s="3" t="b">
@@ -4041,7 +4047,7 @@
       <c r="I101" s="3"/>
     </row>
     <row r="102" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A102" s="32" t="s">
+      <c r="A102" s="28" t="s">
         <v>176</v>
       </c>
       <c r="B102" s="3" t="b">
@@ -4647,7 +4653,7 @@
       <c r="I127" s="3"/>
     </row>
     <row r="128" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A128" s="32" t="s">
+      <c r="A128" s="28" t="s">
         <v>226</v>
       </c>
       <c r="B128" s="3" t="b">
@@ -5040,7 +5046,7 @@
       <c r="I144" s="3"/>
     </row>
     <row r="145" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A145" s="32" t="s">
+      <c r="A145" s="28" t="s">
         <v>257</v>
       </c>
       <c r="B145" s="3" t="b">
@@ -5202,7 +5208,7 @@
       <c r="I152" s="3"/>
     </row>
     <row r="153" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A153" s="32" t="s">
+      <c r="A153" s="28" t="s">
         <v>276</v>
       </c>
       <c r="B153" s="3" t="b">
@@ -5341,7 +5347,7 @@
       <c r="I159" s="3"/>
     </row>
     <row r="160" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A160" s="32" t="s">
+      <c r="A160" s="28" t="s">
         <v>290</v>
       </c>
       <c r="B160" s="3" t="b">
@@ -5967,7 +5973,7 @@
       <c r="I187" s="3"/>
     </row>
     <row r="188" spans="1:9" ht="14.5" x14ac:dyDescent="0.4">
-      <c r="A188" s="32" t="s">
+      <c r="A188" s="28" t="s">
         <v>362</v>
       </c>
       <c r="B188" s="3" t="b">
@@ -6474,7 +6480,7 @@
       <c r="I210" s="3"/>
     </row>
     <row r="211" spans="1:9" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A211" s="32" t="s">
+      <c r="A211" s="28" t="s">
         <v>405</v>
       </c>
       <c r="B211" s="3" t="b">
@@ -15261,6 +15267,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="A6:A32"/>
+    <mergeCell ref="A35:A41"/>
     <mergeCell ref="A44:A54"/>
     <mergeCell ref="A57:A67"/>
     <mergeCell ref="A188:A208"/>
@@ -15272,11 +15283,6 @@
     <mergeCell ref="A145:A150"/>
     <mergeCell ref="A153:A157"/>
     <mergeCell ref="A160:A185"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="A6:A32"/>
-    <mergeCell ref="A35:A41"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>